<commit_message>
Initial commit: neurodegenerative biosensor platform
</commit_message>
<xml_diff>
--- a/alzheimer_pubmed_papers.xlsx
+++ b/alzheimer_pubmed_papers.xlsx
@@ -446,17 +446,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>42768912</t>
+          <t>42775489</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>The Alzheimer's disease risk gene SORL1 is a regulator of excitatory neuronal function.</t>
+          <t>Porous Framework Materials and MXenes as Biosensing Platforms for Amyloid-β Detection.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Alzheimer's &amp; dementia : the journal of the Alzheimer's Association</t>
+          <t>Chemical record (New York, N.Y.)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -466,24 +466,24 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Synaptic dysfunction is an early feature of Alzheimer's disease (AD) and proper localization of proteins involved in pre- and post-synaptic composition is dependent on endosomal recycling and trafficking, cellular processes involving the AD risk gene sortilin-related receptor 1 (SORL1). We examined SORL1's role in synaptic protein composition and neuronal function in human excitatory cortical neurons. Synaptic protein interactions were analyzed using a mesoscale proteomics assay. Immunocytochemistry was used to visualize synaptic proteins and α-amino-3-hydroxy-5-methyl-4-isoxazolepropionic acid receptor subunits. Neuronal function was measured with multi-electrode arrays. Loss of SORL1 expression significantly changes many synaptic protein-protein interactions and patterns of expression. SORL1-deficient neurons exhibit hyperactivity that is primarily amyloid beta independent. SORL1-deficient neurons also have impaired network plasticity. These findings further support a growing body of literature implicating early endosomal recycling defects as drivers of AD pathogenesis.</t>
+          <t>Amyloid-β (Aβ), a 39-43-amino-acid peptide, is closely associated with the pathogenesis of Alzheimer's disease (AD) and undergoes abnormal aggregation that contributes to disease progression. Therefore, rapid and accurate Aβ detection is essential for early AD diagnosis and therapeutic monitoring. Biosensors have emerged as promising analytical tools owing to their simplicity, low cost, high sensitivity, and selectivity. In particular, metal-organic frameworks, covalent organic frameworks, hydrogen-bonded organic frameworks, and MXenes offer unique structural and functional advantages for Aβ sensing. This review summarizes recent advances in Aβ biosensors based on these materials, with emphasis on comparative analytical performance across electrochemical, optical, photoelectrochemical, and dual-mode platforms. Current challenges, including matrix interference, limited discrimination of Aβ isoforms, and biosensor miniaturization, are discussed. Future directions involving artificial intelligence and machine learning are also highlighted to advance rapid, sensitive, and accurate Aβ detection for early AD diagnosis and therapeutic monitoring.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>42768871</t>
+          <t>42772054</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>The Diagnostic Role of FDG-PET in Dementias Presenting with Language and Behavioral Symptom.</t>
+          <t>Next-generation optical biosensors for ultra-early detection of Alzheimer's and Parkinson's diseases: Recent advances, challenges, and future perspectives.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Turk psikiyatri dergisi = Turkish journal of psychiatry</t>
+          <t>Talanta</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -493,24 +493,24 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>This study aimed to assess the diagnostic contribution of Fluorodeoxyglucose Positron Emission Tomography (FDG-PET) in neurodegenerative dementias presenting with language-predominant symptoms, with or without accompanying behavioral changes, and to evaluate the correspondence between PET-derived metabolic patterns and cerebrospinal fluid (CSF) biomarkers. Sixteen patients with language-predominant onset were categorized into two groups: Alzheimer&amp;rsquo;s disease (AD) spectrum (n=8) and the frontotemporal lobar degeneration (FTLD) spectrum (n=8). All participants underwent clinical evaluation, neuropsychological testing, and FDG-PET imaging. Cerebrospinal fluid biomarkers [Amyloid Beta (A&amp;beta;42), total tau, and phosphorylated tau] were analyzed in eligible individuals (n=6). The two groups were compared across demographic, clinical, and neuroimaging parameters. FDG-PET revealed pronounced posterior temporoparietal hypometabolism in AD-spectrum patients, whereas FTLD-spectrum patients demonstrated frontal, insular, and anterior temporal metabolic involvement. Cerebrospinal fluid biomarker profiles consistently supported Alzheimer-type pathology among AD-spectrum cases. In the FTLD group, one patient exhibited borderline-low A&amp;beta;42; however, the corresponding FDG-PET pattern was characteristic of FTLD. FDG-PET demonstrates a supportive role in differentiating AD from FTLD among patients presenting with language-predominant neurodegenerative syndromes. In scenarios where CSF biomarkers are unavailable or yield borderline values, FDG-PET-based metabolic signatures may offer additional guidance and can contribute to strengthening multimodal diagnostic frameworks in geropsychiatry settings.</t>
+          <t>Alzheimer's disease (AD) and Parkinson's disease (PD) are considered among the most difficult neurodegenerative diseases because they are progressive, and there are no reliable tools to make early diagnoses. Traditional diagnostic approaches, such as neuroimaging and CSF analysis, are not ideal for rapid clinical screening and are often invasive and costly. Optical biosensors have become attractive platforms for detecting neurodegenerative markers in recent years, offering ultra-sensitivity and minimal invasiveness. Recent advances in optical biosensing technologies for the early detection of key AD and PD biomarkers, such as amyloid-β, tau protein, α-synuclein, dopamine, and neurofilament light chain (NFL), are highlighted. Several photonic techniques, including fluorescence-based assays, surface plasmon resonance (SPR), surface-enhanced Raman scattering (SERS) and whispering-gallery-mode (WGM) microcavity sensors, are critically described, highlighting their sensing mechanisms, analytical performance, and clinical applications. Significant focus is placed on nanostructured SERS substrates, microfluidically integrated platforms, paper-based optical chips, and WGM microlaser-assisted immunosensors for femtomolar-to-attomolar detection in clinically relevant biofluids. Moreover, the use of sophisticated nanomaterials and artificial intelligence-based data analysis is discussed as an effective approach to developing multiplexed, portable, and point-of-care diagnostics. Finally, the challenges and future directions in translating next-generation optical biosensors for the diagnosis of neurodegenerative diseases are discussed.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>42768868</t>
+          <t>42763160</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Changes in serum β-synuclein precede blood biomarkers of Alzheimer pathology in Down syndrome.</t>
+          <t>Magnetic-assisted catalytic hairpin assembly fluorescent aptasensor for highly sensitive detection of amyloid-beta oligomers as Alzheimer's disease biomarker.</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Alzheimer's &amp; dementia : the journal of the Alzheimer's Association</t>
+          <t>Analytica chimica acta</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -520,24 +520,24 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>There is a need for early, objective markers of Alzheimer's disease (AD)-related synapse dysfunction in adults with Down syndrome (DS). The presynaptic protein β-synuclein is elevated in the blood of adults with DS. This study evaluates the positioning of these changes relative to changes in pathophysiological blood biomarkers along the AD continuum. We quantified serum β-synuclein using immunoprecipitation-mass spectrometry in a cross-sectional cohort (n = 131) spanning the AD continuum in adults with DS (n = 88) and cognitively unimpaired euploid controls (n = 43). β-synuclein levels were elevated in individuals with DS (p &lt; 0.001), preceding symptom onset by two decades and changes in other blood biomarkers (tau phosphorylated at threonine 217, neurofilament light, glial fibrillary acidic protein) by several years. Higher β-synuclein was associated with cortical atrophy (p &lt; 0.001) and hypometabolism (p &lt; 0.001) in AD-vulnerable regions and reduced episodic memory (p &lt; 0.009). These findings consolidate β-synuclein as an early blood-based biomarker of synaptic dysfunction and provide insight into early AD-related mechanisms.</t>
+          <t>The abnormal accumulation of amyloid-beta peptides is a key contributor to Alzheimer's disease. Of these peptides, soluble amyloid-beta oligomers (AβOs) have emerged as potent neurotoxins and early pathological biomarkers. Although AβOs are highly specific biomarkers, their low physiological abundance, structural heterogeneity and matrix interference associated present considerable challenges for conventional diagnostic approaches. Herein, we report a novel fluorescent aptasensor platform for the ultrasensitive detection of AβOs. The platform integrates magnetic preconcentration with a signal amplification strategy based on catalytic hairpin assembly (CHA). To achieve simultaneous selective recognition of AβOs and efficient CHA initiation, magnetic beads were functionalized with rationally designed double-stranded DNA complexes, which were formed through the hybridization of an AβO-specific aptamer and a CHA-initiator fragment. Upon the specific binding of AβOs, the AβO-specific aptamer competitively dissociates from the magnetic beads, thereby unmasking the surface-tethered initiator to trigger the CHA circuit. The circularly generated CHA products serve as a self-amplifying signal indicator, whereas the magnetic beads enhance target-capturing capacity and facilitate the removal of complex matrix interferences prior to amplification. Experimental results revealed that the proposed system exhibited a broad linear detection range from 10 pg mL These findings demonstrate the potential of integrating aptamer-mediated magnetic capture with CHA-driven signal amplification for ultrasensitive AβO detection. The spatial separation of AβO-aptamer binding and CHA amplification through magnetic beads effectively minimizes matrix interference while permitting large sample volumes. This strategy has the potential to serve as sensitive tool for early Alzheimer's disease diagnosis.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>42768866</t>
+          <t>42721512</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Unmasking preclinical Alzheimer's pathology: auditory distraction cost and occupational reserve jointly discriminate amyloid positivity in subjective cognitive decline.</t>
+          <t>Affinity peptide-based microfluidic electrochemical system for ultrasensitive detection of amyloid-β peptides.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Alzheimer's &amp; dementia : the journal of the Alzheimer's Association</t>
+          <t>Biosensors &amp; bioelectronics</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -547,24 +547,24 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Conventional cognitive instruments exhibit limited efficacy in detecting insidious cognitive decline in subjective cognitive decline (SCD) due to neural compensation. We hypothesized that auditory distraction during a visual memory task would unmask preclinical amyloid beta (Aβ) vulnerability. We evaluated 112 participants (SCD and mild cognitive impairment [MCI]) using the MemTrax test under quiet and noisy conditions to quantify distraction costs (d-MTxc). Aβ status and cognitive reserve were assessed via positron emission tomography and the Cognitive Reserve Index questionnaire (CRIq). Aβ-positive SCD individuals performed normally in quiet but showed higher d-MTxc than Aβ-negative peers (11.17 ± 5.762 vs 6.67 ± 5.096). Higher CRIq-WorkingActivity (CRIW) scores identified Aβ positivity and moderated performance. The combination of d-MTxc and CRIW accurately classified Aβ positivity (AUC = 0.836), whereas MCI individuals exhibited metabolic network fragmentation. Auditory distraction taxes cognitive capacity to expose compensatory failures coupled with Aβ burden. This paradigm, interacting with occupational reserve, offers a promising digital biomarker framework for preclinical Alzheimer's screening.</t>
+          <t>The early diagnosis of Alzheimer's disease (AD) urgently requires analytical tools that simultaneously provide ultrahigh sensitivity, specific recognition, and fully automated operation to detect low-abundance amyloid-β (Aβ) peptides in peripheral blood. To address this challenge, an affinity peptide (AP)-based microfluidic electrochemical system (μF-APEC) was developed. As the core recognition elements in a sandwich assay, the APs were selected from a phage display library with a diversity of 100 billion variants, enabling high-affinity binding and precise recognition. By integrating the electrochemical biosensor with a microfluidic chip, the μF-APEC system enables automated sample injection, on-chip mixing, and electrochemical readout, with the entire detection process completed in less than 20 min. Under the optimized detection conditions, the system achieved ultrasensitive quantification, with limits of detection of 38 fg/mL for Aβ40 and 14 fg/mL for Aβ42, with a linear range of 100 fg/mL to 1 ng/mL. In serum samples, the μF-APEC system showed strong agreement with conventional enzyme-linked immunosorbent assay measurements and clearly distinguished AD patients from healthy individuals. By combining AP-based specific recognition with high sensitivity and automated operation, the μF-APEC system provides a robust and practical platform for the detection of low-abundance peripheral Aβ peptides, demonstrating its potential for the early screening of AD.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>42768864</t>
+          <t>42716046</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Enhancing early Alzheimer's disease clinical trials through prognostic score covariate adjustment.</t>
+          <t>Neuroimaging in the era of biologically defined Alzheimer's disease and disease-modifying therapy.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Alzheimer's &amp; dementia : the journal of the Alzheimer's Association</t>
+          <t>The Lancet. Neurology</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -574,24 +574,24 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>A prognostic score (PS) summarizes a patient's expected disease progression and can increase the statistical efficiency of clinical trials when included as an analysis covariate. We pooled patient data from observational studies and randomized trials for early Alzheimer's disease (AD) and trained PS candidates to predict 18-month changes in the Clinical Dementia Rating Scale - Sum of Boxes (CDR-SB) score. The efficiency gains achieved through covariate adjustment were evaluated in a held-out trial (N = 650). A machine learning PS achieved a Pearson correlation of 0.48 between predicted and observed CDR-SB changes in an internal test set (N = 398). Adjusting for this PS in the held-out trial increased power from 80% to 87.9% (95% confidence interval [CI]: 85.5%-90.2%) with the original sample size. Alternatively, this approach could reduce the required sample size by 19.7% (95% CI: 13.7%-25.7%) while maintaining 80% power. Our findings support the use of PS adjustment for enhancing the efficiency of early AD trials.</t>
+          <t>Disease-modifying therapies and biomarker-based diagnostic frameworks will fundamentally altered the clinical diagnosis and management of Alzheimer's disease. Diagnosis is increasingly anchored in the biological evidence of pathology rather than clinical presentation alone, with implications for treatment eligibility, prognosis, and monitoring. In clinical practice, patients with memory complaints can present with complex mixed pathologies that develop across the lifespan. Brain imaging, particularly MRI and PET, plays a crucial role in visualising these cumulative abnormalities. With Alzheimer's disease-specific therapies now available in many regions of the world, amyloid PET plays a central role in establishing Alzheimer's disease diagnosis, determining eligibility for amyloid-targeting therapies, and quantifying treatment-related amyloid clearance. In settings where available, tau PET informs biological stage, prognosis, and clinical heterogeneity. MRI remains indispensable for differential diagnosis, the assessment of comorbid and vascular pathology, and monitoring for complications, particularly amyloid-related imaging abnormalities. Technological advances-including quantitative imaging, artificial intelligence, accelerated acquisition, and workflow optimisation-are improving reliability, efficiency, and access to these tools. Neuroimaging is now a cornerstone of Alzheimer's disease care and a crucial discriminator tool for characterising brain injury across the lifespan. With emerging fluid biomarkers, neuroimaging supports accurate diagnosis, prognosis, and treatment monitoring.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>42768849</t>
+          <t>42716045</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Comparative Risk of Nonarteritic Anterior Ischemic Optic Neuropathy Among Glucagon-Like Peptide-1 Receptor Agonists: An Integrated Safety and Mechanistic Analysis.</t>
+          <t>Fluid biomarkers in the evolving care landscape of Alzheimer's disease and related disorders.</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Diabetes, obesity &amp; metabolism</t>
+          <t>The Lancet. Neurology</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -601,24 +601,24 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Glucagon-like peptide-1 receptor agonists (GLP-1RAs) are widely used for Type 2 diabetes (T2DM) and obesity, but emerging evidence links them to nonarteritic anterior ischemic optic neuropathy (NAION). Whether this risk differs across agents and the underlying mechanisms remains unclear. We aimed to compare the risks of NAION associated with different GLP-1RAs and to explore the potential molecular mechanisms underlying this adverse reaction. A network meta-analysis was performed to quantitatively compare the differences in NAION risk. Real-world pharmacovigilance data from the FDA Adverse Event Reporting System (FAERS) were used for validation. Network toxicology was further applied to identify central hub targets and signalling pathways. Molecular docking was conducted to evaluate the binding capacity of GLP-1RAs to central hub targets. The network meta-analysis revealed significant differences in NAION risk across GLP-1RAs. Compared with non-GLP-1RA treatments, semaglutide showed the highest risk (HR = 1.538, 95% CI: 1.305-1.816), followed by liraglutide (HR = 1.251, 95% CI: 1.080-1.450). FAERS pharmacovigilance analysis suggested a strong disproportionate signal for semaglutide (ROR = 94.534, 95% CI: 83.093-107.552) and a statistically significant but weaker signal for liraglutide (ROR = 4.519, 95% CI: 2.617-7.802). Network toxicology identified CASP3 as the central hub target, and pathway enrichment analysis revealed that the underlying mechanisms were primarily related to Alzheimer's disease, neurodegeneration pathways, and lipid and atherosclerosis pathways. Molecular docking suggested that semaglutide and liraglutide had high binding affinity to CASP3. The combined strategy of network meta-analysis, pharmacovigilance, network toxicology and molecular docking provides insights into possible risk differences and potential mechanisms, and may guide future research on the safety profile of GLP-1RAs.</t>
+          <t>Fluid biomarkers for Alzheimer's disease have advanced rapidly during the past several years driven by breakthroughs including development of ultrasensitive and multiplexing technologies and high specificity antibodies. Blood-based biomarkers, such as neurofilament light for frontotemporal dementia and amyotrophic lateral sclerosis, and phosphorylated tau 217 for the diagnosis of Alzheimer's disease, are now being implemented in clinical practice, which is particularly timely because of the increasing clinical availability of amyloid-targeting treatments in Alzheimer's disease. Multiple fluid biomarkers are needed to capture the complexity of disease mechanisms for precise diagnosis and to measure the diverse pathologies that lead to dementia, such as vascular, α-synuclein, and TDP-43 pathologies. Moreover, fluid biomarkers can aid in capturing heterogeneity in treatment course between patients, probably due to copathologies or key intermediates, including microglia and astrocyte dysregulation. Increased focus on biomarker-pathology relationships in experimental models will likely accelerate biomarker development and further the understanding of their precise substrates. Future clinical implementation of biomarkers to capture the full complexity of pathologies will likely be facilitated by the expansion of diagnostic methods, development of point of care technologies, and remote sampling approaches.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>42768846</t>
+          <t>42715723</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Do amyloid trajectories reach a ceiling? Evidence from iterative approximation and simulation.</t>
+          <t>DNA- and aptamer-based biosensors for Alzheimer's disease biomarkers toward clinical translation.</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Alzheimer's &amp; dementia : the journal of the Alzheimer's Association</t>
+          <t>Talanta</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -628,24 +628,24 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Qualitative models of Alzheimer's disease (AD) pathology often posit that amyloid accumulation follows a sigmoid curve, indicating that the rate of deposition wanes over time. Longitudinal positron emission tomography (PET) data now allow us to investigate amyloid accumulation trajectories with greater detail and over longer follow-up periods. We combine inferences from simulated amyloid trajectories, empirical PET data from the Alzheimer's Disease Neuroimaging Initiative (ADNI), and the sampled iterative local approximation algorithm (SILA) to assess whether amyloid accumulation reaches a physiologic ceiling. SILA reliably detects a ceiling in simulated scenarios that impose a sigmoid shape. Fit to ADNI, SILA does not appear to indicate the presence of a ceiling. Amyloid trajectories may not reach a physiologic ceiling during the stages of AD typically observed while patients remain under follow-up in cohort studies. Illustrative models of biomarker cascades, while useful for conceptualizing pathologic processes, may not represent amyloid trajectory shapes accurately.</t>
+          <t>Alzheimer's disease (AD) is a progressive neurodegenerative disorder for which early diagnosis remains a major challenge. DNA-based biosensors and aptamer-based biosensors have emerged as complementary platforms for the sensitive and selective detection of Alzheimer's disease biomarkers. DNA biosensors primarily detect nucleic acid biomarkers, including disease-associated microRNAs, through sequence-specific hybridization, whereas aptamer-based biosensors are mainly employed for the recognition of protein biomarkers such as amyloid-β and tau proteins. Recent advances in nanomaterials have significantly enhanced biosensor performance by improving target recognition, signal amplification, and analytical sensitivity. This review summarizes recent developments in both DNA hybridization-based biosensors and aptamer-based biosensors for Alzheimer's disease biomarkers, highlighting their distinct recognition mechanisms, sensing strategies, and applications in electrochemical, optical, fluorescence, and nanomaterial-assisted platforms. Representative systems are compared in terms of analytical performance, detection limit, selectivity, and applicability to biological samples. Current challenges related to reproducibility, matrix interference, standardization, and clinical validation are also discussed. Despite remarkable progress, further efforts are required to translate these technologies into robust and reliable point-of-care diagnostic tools. The integration of advanced nanomaterials, DNA nanotechnology, and multiplexed sensing platforms is expected to accelerate the clinical implementation of biosensors for early AD diagnosis.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>42768750</t>
+          <t>42705087</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Catestatin peptide ameliorates tauopathy and amyloidogenesis via adrenergic inhibition.</t>
+          <t>A signal-locked clamped hybridization chain reaction nanoamplifier for rapid and highly sensitive analysis of Aβ42.</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Molecular therapy : the journal of the American Society of Gene Therapy</t>
+          <t>Talanta</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -655,24 +655,24 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Neurodegenerative disorders such as Alzheimer's disease (AD), Corticobasal Degeneration (CBD), and Progressive Supranuclear Palsy (PSP) are characterized by tau aggregation, neuroinflammation, and progressive cognitive decline. Although metabolic dysregulation and neuropeptide imbalance have been linked to these disorders, the functional consequences of this imbalance and its reversal remain poorly understood. Our previous work identified chromogranin A (CgA), the gene encoding a pro-hormone for several metabolic peptides, as a key regulator of tau pathology. Here, we investigate Catestatin (CST), a CgA-derived peptide, for its role in modulating tauopathy. We report marked reductions in CST levels and an increase in Pancreastatin (PST) in the hippocampus and cortex of AD brains, as well as in the frontal cortex of CBD and the basal ganglia of PSP. CST-supplementation in cortical neuronal cultures and organotypic slice cultures (OTSC) reduced Tau phosphorylation and aggregation. In vivo, CST administration to PS19 tauopathy mice decreased pathological Tau species, attenuated gliosis, improved cognitive function, and reduced amyloid burden and neuroinflammation in 5xFAD mice. Mechanistically, CST reduced epinephrine levels in PS19 and 5xFAD mice, suppressed Protein Kinase A hyperactivation in PS19 and OTSC, and revealed a link between CST deficiency, adrenergic stress signaling, tauopathy-mediated neurodegeneration, and the therapeutic potential of CST supplement.</t>
+          <t>Amyloid-beta 42 (Aβ42) is a core biomarker associated with Alzheimer's disease (AD), but accurate quantification of low-abundance plasma Aβ42 remains challenging because of matrix interference, limited assay sensitivity, and time-consuming procedures in conventional methods. Herein, we developed an enzyme-free fluorescence biosensing platform integrating a triple-helix aptamer probe (THAP) with clamped hybridization chain reaction (cHCR), termed T-cHCR, for sensitive Aβ42 analysis. In this system, Aβ42 recognition induces controlled release of a trigger probe from the triplex-locked THAP module, which subsequently initiates a two-hairpin cHCR cascade for low-background signal amplification. Under optimized conditions, the T-cHCR assay exhibited a linear response to Aβ42 from 1 to 1000 pg/mL with a limit of detection of 1.16 pg/mL, showing an 8.1-fold lower LOD than the manufacturer-reported minimum detectable dose of the ELISA kit used in this study. The assay also displayed acceptable specificity, reproducibility, and storage stability. Preliminary analysis of clinical plasma samples showed significantly different Aβ42 levels between AD patients and age-matched healthy controls, supporting the potential of T-cHCR for further validation in plasma AD biomarker analysis. Overall, this integrated THAP-cHCR strategy provides a rapid, enzyme-free, and low-background approach for ultrasensitive plasma Aβ42 detection.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>42768736</t>
+          <t>42702988</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Fluid Intelligence and Executive Dysfunction in Progressive Supranuclear Palsy.</t>
+          <t>High-Performance Screen-Printed OECT-Inspired with Encased Cassette Based on PEDOT:GO for Sensitive and Specific Electrochemical Aptasensing of Aβ-42 in Management of Alzheimer's Disease.</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Movement disorders clinical practice</t>
+          <t>ACS applied bio materials</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -682,24 +682,24 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Fluid intelligence (g) contributes to executive-task performance, but its role in progressive supranuclear palsy (PSP) remains unclear. To examine whether executive deficits in PSP are explained by reductions in g. Thirty-five PSP patients, 39 Parkinson's disease (PD) patients and 18 healthy controls underwent neuropsychological assessment. G was derived using principal component analysis from non-executive cognitive measures. Group differences in executive performance were examined before and after controlling for g. Healthy controls provided contextual comparison. In PSP versus PD, differences in phonemic fluency and TMT-B were no longer significant after controlling for g, whereas WCST categories remained significant. In PSP versus healthy controls, WCST and phonemic fluency remained significant after controlling for g. Sensitivity analyses in cognitively preserved participants showed similar results. Executive deficits in PSP are partly associated with reduced g, but cognitive flexibility appears to reflect an additional disease-related impairment.</t>
+          <t>Recently, substantial interest has emerged in developing point-of-care diagnostic devices for Alzheimer's disease (AD), a progressive neurodegenerative disorder characterized by the accumulation of beta-amyloid (Aβ1-42) peptides that act as critical biomarkers for early detection. In response to the growing demand for noninvasive and accessible diagnostic tools, this study presents a highly sensitive organic electrochemical transistor-inspired biosensor for the detection of Aβ-42 in saliva. The device is based on a paper substrate modified with a PEDOT:GO composite and a Ag-Au nanocomposite, which together enhance electrical conductivity and improve the electrochemical response. A highly selective Aβ1-42-binding aptamer is immobilized on the sensor surface. This platform enables real-time signal amplification, allowing the detection of Aβ-42 over a dynamic range of 1 pg/mL to 10 μg/mL. This biosensor demonstrates excellent sensitivity, selectivity, and reproducibility, making it a potential tool for noninvasive, point-of-care detection. The use of artificial saliva as a diagnostic medium further enhances its applicability for early screening, especially in decentralized or resource-limited healthcare environments.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>42768715</t>
+          <t>42696024</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Non-motor symptoms questionnaire-based profiles in early-stage dementias: A prospective cohort study.</t>
+          <t>Simultaneous Detection of Dopamine and Xanthine in Human Sweat by Ultrasensitive MoB-MBene/PVA Sponge-like Hydrogel Grown on a Porous Nickel Substrate.</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Journal of Alzheimer's disease : JAD</t>
+          <t>ACS applied bio materials</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -709,24 +709,24 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">BackgroundCurrent knowledge regarding the nature and prevalence of non-motor symptoms across different types of dementia is limited. While Alzheimer's disease (AD), behavioral variant frontotemporal dementia (bvFTD), and dementia with Lewy bodies (DLB) are primarily characterized by cognitive and motor symptoms, several other features such as non-motor symptoms are also known to occur in all these conditions.ObjectiveTo assess non-motor symptoms in early-stage dementia and characterize symptom profiles across different neurodegenerative dementia diseases.MethodsA total of 64 AD, 38 bvFTD, and 17 DLB early-stage patients, along 63 cognitively healthy controls (HC), were prospectively recruited from Kuopio and Oulu University Hospitals. Non-motor symptoms were evaluated using the Non-Motor Symptoms Questionnaire (NMSQ), focusing on gastrointestinal, neuropsychiatric, cognitive, sleep-related and sensory-motor domains within three timeframes prior to the baseline visit.ResultsDLB patients exhibited the highest prevalence of non-motor symptoms across all domains. bvFTD and AD patients did not show disease group specific symptoms, but apathy and paranoidal thoughts appeared earlier in bvFTD than AD or DLB. Diplopia was reported by 14% of DLB patients (Fisher exact test, </t>
+          <t>Dopamine and xanthine are essential biomolecules for neurological disorders and oxidative stress, respectively, and their abnormal concentrations are associated with Parkinson's disease, schizophrenia, Alzheimer's disease, and renal dysfunction. To overcome the limitations of invasive conventional diagnostics, a flexible MoB/PVA hydrogel on nickel foam is fabricated for the simultaneous, non-invasive electrochemical detection of dopamine and xanthine in human sweat. It is prepared through selective alkali etching and solvothermal synthesis. Characterization of the optimized MoB-MBene hydrogel (7 wt %), such as FTIR, confirms characteristic Mo-B vibrational bands, while SEM analysis reveals a sponge-like porous morphology favorable for rapid ion transport and enhanced electroactive sites. Using the DPV technique, the MoB/PVA hydrogel/NF sensor, which has a higher active surface area, demonstrates the simultaneous detection of dopamine, with a linear range from 50 nM to 500 μM, detection limit of 0.35 nM, and sensitivity of 158 μA nM-1 cm-2, and xanthine, with a linear range of 100 nM to 1 mM, detection limit of 0.098 nM, and sensitivity of 95.2 μA nM-1 cm-2, with a peak separation (ΔEp) of 285 mV. The superior electrochemical performance is attributed to the synergistic effect arising from abundant active sites in the ion-rich MoB/PVA hydrogel, facilitating higher charge-transfer kinetics and resulting in enhanced peak currents and well-resolved peaks for simultaneous sensing with 99.6-101.3% recovery for dopamine and 99.3-101.4% recovery for xanthine. Repeatability tests (N = 4) yielded dopamine with a 0.6% RSD and xanthine with a 1.93% RSD. The flexible sensor exhibits excellent selectivity and stability for up to 4 weeks and holds potential for point-of-care and flexible wearable devices.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>42768280</t>
+          <t>42683894</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Reject Option for Medical Image Classification Using CNN-Derived Latent-Space Neighbourhood Analysis.</t>
+          <t>Toward harmonized reporting of Alzheimer's disease biomarkers in clinical practice.</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Journal of imaging informatics in medicine</t>
+          <t>Clinical chemistry and laboratory medicine</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -736,24 +736,24 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reliable uncertainty estimation is a key requirement for the clinical adoption of convolutional neural networks (CNNs) in biomedical imaging. We propose a reject option framework that assesses prediction reliability by leveraging the local structure of the latent space. The method is based on three latent-space features: Simple Data Point Target Density ( </t>
+          <t>Cerebrospinal fluid biomarkers, and more recently blood-based biomarkers, are playing a pivotal role in reshaping the clinical management of neurodegenerative diseases, supporting early detection, biological diagnosis, patient stratification, prognostic assessment, therapeutic decision-making, and longitudinal disease monitoring. To effectively support clinical decision-making, biomarker measurements must be communicated in a standardized, transparent, and clinically interpretable manner. Despite international quality standards, considerable heterogeneity persists in reporting practices, including differences in terminology, units of measurement, analytical descriptions, reference frameworks, and interpretative comments, limiting comparability across laboratories and potentially affecting clinical decision-making. In this article, we discuss the principles of harmonized reporting for Alzheimer's disease biomarkers and propose a structured framework for standardized clinical neurochemistry reports. We describe the essential components of a harmonized report, including report identification, analytical information, specification of analytical method and platform, standardized units of measurement, appropriate use of reference intervals and clinical decision thresholds, documentation of pre-analytical and quality-related factors, and evidence-based interpretative comments. We further discuss the importance of structured multimarker interpretation and the need to contextualize biomarker findings within the clinical scenario. Finally, we examine the role of harmonized reporting in promoting interoperability across healthcare systems, facilitating longitudinal patient monitoring, supporting electronic health records and standardized terminologies, and enabling artificial intelligence-driven clinical decision support. As neurodegenerative disease diagnostics continue to evolve and novel biomarkers and technologies emerge, harmonized reporting should be regarded as a critical component of laboratory quality, ensuring that analytical advances translate into consistent, clinically meaningful, and interoperable information that ultimately improves patient care.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>42768200</t>
+          <t>42678362</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Tinosinenside A ameliorates Alzheimer's disease-related pathology in APP/PS1 mice, accompanied by reduced neuroinflammation and altered microglial phenotype-associated marker expression.</t>
+          <t>A sandwich ECL immunoassay system for tau protein detection using Ru(II)-AuNP signal probes integrated with copper nanoclusters.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Naunyn-Schmiedeberg's archives of pharmacology</t>
+          <t>Analytical methods : advancing methods and applications</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -763,24 +763,24 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Tinospora sinensis (Lour.) Merr. has traditionally been used for its anti-inflammatory properties. Tinosinenside A (Tis A), a major sesquiterpene glycoside isolated from this plant, has shown neuroprotective activity; however, its effects on Alzheimer's disease (AD)-related neuroinflammation remain unclear. This study evaluated the effects of Tis A on behavioral impairment, neuroinflammation, and amyloid-β (Aβ) pathology in APPswe/PSEN1dE9 (APP/PS1) mice. APP/PS1 mice received oral Tis A for 6 months and were evaluated at 11 months of age using behavioral, histopathological, biochemical, and molecular analyses. Tis A partially improved behavioral performance, reduced Aβ plaque burden and pro-inflammatory cytokine levels, attenuated microglial overactivation, shifted microglial phenotype-associated marker expression toward a less pro-inflammatory profile, and alleviated neuronal apoptosis and histopathological damage. These effects were accompanied by reduced TLR4 and NLRP3 inflammasome-related protein expression and decreased phosphorylation of NF-κB p65 and IκBα. Collectively, these findings indicate that Tis A attenuates neuroinflammation and AD-related neuropathology while providing partial behavioral benefits in APP/PS1 mice, supporting its further investigation as a natural-product-derived therapeutic lead for AD.</t>
+          <t>Tau protein is an important biomarker which is associated with neurodegenerative disorders, particularly Alzheimer's disease, where abnormal tau aggregation and hyperphosphorylation contribute to neuronal dysfunction and cognitive decline. The sensitive and early detection of tau protein is therefore crucial for the diagnosis, prognosis and therapeutic monitoring of neurodegenerative diseases. Owing to its clinical significance, the development of rapid, highly sensitive and reliable analytical platforms for tau detection has gained considerable attention in biomedical diagnostics. In this work, a Ru(II) based homogeneous sandwich ECL immunosensor was developed for the turn-on detection of tau. A polyclonal antibody was conjugated with Ru(II)@AuNP, which served as the ECL signal probe, and further integrated with monoclonal antibody conjugated L-Cys-CuNC to construct the ECL immunoassay system. Upon the addition of tau protein, the ECL intensity was enhanced due to the specific antigen-antibody interaction. The probe is selective and sensitive towards tau with a limit of detection of 0.23 pg mL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>42768165</t>
+          <t>42676313</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Multimodal prediction of MCI-to-dementia conversion over a two-year window.</t>
+          <t>Colorimetric gold nanosensors for monitoring protein aggregation: implications for Alzheimer's disease.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>GeroScience</t>
+          <t>Chemical communications (Cambridge, England)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -790,24 +790,24 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Mild cognitive impairment (MCI) represents a heterogeneous clinical state where some individuals remain stable while others progress to dementia. Identification of patients who are at high risk for near-term conversion remains a critical challenge for timely intervention. We developed an explainable multimodal machine-learning framework to predict progression from MCI to dementia within a clinically meaningful two-year period. We analyzed 2008 samples from 828 unique MCI subjects from the Alzheimer's Disease Neuroimaging Initiative (ADNI), including cognitive/functional assessments, demographic/genetic variables, and structural MRI features. Subjects were classified as stable MCI (sMCI, n = 1306) or progressive MCI (pMCI, n = 702) based on two-year outcomes. Machine learning algorithms were evaluated on unimodal and multimodal using nested cross-validation, and explainability was assessed using SHapley Additive exPlanations (SHAP) and permutation feature importance. The combination of cognitive assessments, demographics/risk factors and structural MRI features outperformed individual modalities, highlighting the complementary relationship between cognitive-functional decline and neuroanatomical degeneration. The best-performing model, a calibrated XGBoost, achieved a balanced accuracy of 81.28% ± 2.56% during cross-validation and 81.99% (bootstrap mean 81.97%, 95% CI: [78.22%-85.51%]) on an independent held-out test set. Explainable AI analyses identified functional impairment measures (Functional Activities Questionnaire, Clinical Dementia Rating - Sum of Boxes), cognitive performance scores (Alzheimer's Disease Assessment Scale - Cognitive Subscale 11-item version, Alzheimer's Disease Assessment Scale - Cognitive Subscale 13-item version, Mental State Examination), APOE ε4 status, and structural abnormalities within the hippocampus, lateral ventricle, parietal and temporal regions, and amygdala, as the most influential predictors of conversion. Short-term progression from MCI to dementia can be predicted with high accuracy using multimodal information obtained from a single clinical visit. The convergence of cognitive impairment and region-specific neurodegeneration emerged as the strongest indicator of conversion risk.</t>
+          <t>Alzheimer's disease (AD) is the leading cause of dementia worldwide. It remains a major public health challenge due to the lack of early diagnostic tools and effective disease-modifying therapies. Molecularly, AD is characterized by extracellular amyloid-β (Aβ) plaques and intracellular Tau tangles, as well as soluble oligomers that are likely the neurotoxic species. However, the transient and heterogeneous nature of these oligomers makes them difficult to detect using conventional biosensing approaches. Nanomaterial-based colorimetric biosensors have emerged as promising platforms for detecting protein aggregates and discovering aggregation inhibitors. Specifically, the localized surface plasmon resonance properties of metallic nanomaterials can enable rapid, label-free, and visually detectable colorimetric sensing of molecular interactions. These features can be leveraged to monitor protein aggregation processes in real time and achieve high-throughput screening of aggregation inhibitors, which may collectively enable early detection and timely intervention of AD progression. This Review Article presents the design and engineering of gold-nanomaterial-based colorimetric biosensors for monitoring protein aggregation and highlights the current challenges and emerging opportunities for applying these nanosensors to combat AD.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>42768129</t>
+          <t>42657615</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>A multi-omics insight into the sex-specific burden of tobacco-associated neurodegeneration: trends, projections, and mechanistic clues from the TH gene.</t>
+          <t>Quantification of Phosphorylated Tau Protein in Alzheimer's Disease Patients' Fluids With Electrolyte-Gated Organic Transistor Biosensors.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Neurological sciences : official journal of the Italian Neurological Society and of the Italian Society of Clinical Neurophysiology</t>
+          <t>Advanced healthcare materials</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -817,24 +817,24 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Tobacco exposure significantly influences neurological health, yet its specific associations with Parkinson's disease (PD) and Alzheimer's disease and other dementias (ADOD), including mechanisms, require clarification. Using data from the Global Burden of Disease (GBD) 2021 study, multidimensional stratified comparisons of global PD and ADOD attributable to tobacco exposure were performed across dimensions including sex, socio-demographic index (SDI) quintiles, GBD sub-regions, and national levels. Furthermore, autoregressive integrated moving average and exponential smoothing models were incorporated to project trends until 2050. Bioinformatics analysis was conducted to identify key genes linking nicotine metabolism and sex differences. Tobacco exposure exerted a negative modulatory effect on PD burden but increased ADOD risk. Marked sex-specific differences existed, with males more affected. Regional heterogeneity was pronounced: PD impact was strongest in East Asia, while ADOD burden was highest in high-SDI regions. Projections showed rising ASRs for males but a decline for females. Mechanistically, the TH gene was a key nexus connecting PD, nicotine pathways, and sex differences, potentially explaining the stronger effect in males. Tobacco exposure differentially influences PD and ADOD, with distinct patterns by sex and region. It is detrimental for ADOD but may negatively modulate PD. The burden is projected to increase over the next three decades with persistent sex disparities. The TH gene may provides a mechanistic clue for the sex-heterogeneous effect against PD.</t>
+          <t>Dementia is a syndrome that affects millions of people in the world, and Alzheimer's disease (AD) is the most common cause. The diagnosis of AD begins with cognitive symptoms such as mild cognitive impairment (MCI) but requires the demonstration and quantification of the underlying neuropathological processes through the measurement of specific biomarkers. Among these, the phosphorylated tau protein at threonine 181 (p-tau 181) is considered specific for AD diagnosis in people with MCI. In this work, we report the detection of p-tau 181 spanning from physiological to pathological concentrations in cerebrospinal fluids from patients with MCI. The proposed sensor is based on an electrolyte-gated organic transistor functionalized with specific anti-p-tau 181 antibodies. We analyzed the multiparametric sensor response using a Langmuir model to extract the thermodynamic affinity constant, resulting in values between 10</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>42767982</t>
+          <t>42648826</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Post mortem MRI of cholinergic white matter pathways across neurodegenerative diseases.</t>
+          <t>Multiplexed EDL-FET biosensor with tannic acid stabilization for simultaneous p-Tau217 and Aβ</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Alzheimer's &amp; dementia : the journal of the Alzheimer's Association</t>
+          <t>Analytica chimica acta</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -844,24 +844,24 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Cholinergic white matter pathway (CWMP) degeneration is central in Alzheimer's disease (AD) and Lewy body disease (LBD). CWMP degeneration can be assessed in vivo using magnetic resonance imaging (MRI) proxies, but neuropathological validation is limited. We studied post mortem in situ 3T MRIs of 55 brain donors with standardized neuropathologic assessment (AD, LBD, AD+LBD, other dementias, controls). CWMP integrity was assessed quantitatively using diffusion tensor imaging and visually using the Cholinergic Pathways Hyperintensities Scale (CHIPS) on fluid-attenuated inversion recovery MRI. CWMP diffusivity was strongly associated with CHIPS (p &lt; 0.001), independent of global white matter damage. AD and AD+LBD showed greater CWMP degeneration than LBD, other dementias, and controls (p &lt; 0.05). Multivariate analyses across neuropathological variables identified hippocampal sclerosis and vascular co-pathology as strongest predictors for CWMP degeneration. CWMP degeneration is pronounced in AD and mixed AD+LBD pathology and is additionally affected by vascular co-pathology and hippocampal sclerosis. CHIPS may serve as a clinically accessible MRI-based proxy of CWMP integrity.</t>
+          <t>Alzheimer's disease (AD) is a leading cause of disability in aging societies, underscoring the need for practical blood-based biomarker assays. Stroke patients face an elevated risk of AD-related cognitive impairment, yet reliable, scalable tools for early biomarker assessment in this population remain lacking. Current platforms are limited by low throughput, instability, and demanding sample preparation that restricts point-of-care translation. This study addresses the need for a multiplexed, clinically practical biosensor capable of simultaneously measuring AD-relevant biomarkers in both plasma and whole blood. An eight-channel electric double-layer field-effect transistor (EDL-FET) platform was developed to simultaneously measure phosphorylated tau (p-tau217) and the Aβ</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>42767917</t>
+          <t>42648363</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Nanoconjugation of chalcone derivatives and carbon nitride dots for the inhibition of tau aggregation.</t>
+          <t>Endolysosomal inhibition uncouples tau uptake from intracellular seeding.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Colloids and surfaces. B, Biointerfaces</t>
+          <t>The Journal of biological chemistry</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -871,24 +871,24 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Tau aggregation is a pathological hallmark of Alzheimer's disease, yet small-molecule inhibitors targeting this process often face limitations in solubility, selectivity, and bioavailability. In this study, we engineered a library of hybrid nanostructures by covalently conjugating eleven structurally diverse chalcone derivatives to carbon nitride dots (CNDs), aiming to enhance their physicochemical stability and therapeutic efficacy. The resulting CND-chalcone conjugates exhibited favorable aqueous dispersibility and minimal cytotoxicity in HEK293 and HeLa cells. In vitro aggregation assays revealed that the conjugates modulated tau fibrillization in a structure-dependent manner, with several hybrids, particularly those containing hydroxyl or selectively positioned methoxy groups, showing strong inhibitory effects. Thioflavin-T fluorescence assays confirmed that the most active conjugates disrupted both nucleation and elongation phases of fibril formation. Notably, one hybrid (CNDs-S6) outperformed its free chalcone counterpart, suggesting synergistic interactions between the nanoparticle platform and ligand. These findings highlight the potential of CND-chalcone architectures as multifunctional nanoinhibitors and offer a rational approach to designing aggregation-targeting nanotherapeutics for neurodegenerative disease intervention.</t>
+          <t>Neurodegenerative tauopathies, including Alzheimer's disease, appear to be driven by propagation of tau assemblies, which must access the cytoplasm to recruit monomer and self-replicate, a process termed "seeding." The prevailing model holds that tau seeds enter cells via macropinocytosis and reach the cytosol through lysosomal rupture or micro-perforation. Our findings revise this model by revealing that endocytosis is not required for seeding. Using genome-scale CRISPR screening, we identified multiple v-ATPase components whose loss reduced tau uptake (measured by flow cytometry) yet paradoxically increased seeding (measured by FRET biosensors). Acute v-ATPase inhibition with bafilomycin A1 produced the same effect in v2L tau biosensors and iPSC-derived neurons. Among regulators of endosome maturation, dominant-negative Rab5a decreased internalization while enhancing cytoplasmic templating. Cholesterol depletion produced identical results. Strikingly, transient hypothermia eliminated virtually all detectable tau uptake and dramatically increased seeding, without affecting subsequent tau monomer or aggregate degradation. We conclude that efficient endolysosomal trafficking does not appear to be required for cytoplasmic seeding under the conditions studied here. Across diverse perturbations, reduced endolysosomal flux consistently enhanced tau seeding, consistent with prior work indicating that most internalized aggregates are routed toward degradation rather than amplification. To seed effectively, tau must cross the plasma or vesicular membranes into the cytoplasm. We have found that proper endolysosomal trafficking suppresses cytoplasmic tau seeding, as all perturbations augmented this process. These findings reframe the role of the endolysosomal system in tau seeding and identify membrane transit rather than macropinocytosis itself as a critical gateway to cytoplasmic tau amplification.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>42767717</t>
+          <t>42645045</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Running out the clock: Circadian rhythm dysfunction in cognitive disease.</t>
+          <t>Progress in Optical Methods for the Detection of Two Core Blood Biomarkers of Alzheimer's Disease: Amyloid-Beta and Tau Proteins.</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>International review of neurobiology</t>
+          <t>Biosensors</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -898,24 +898,24 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Lifespan is increasing such that within a few decades approximately twenty percent of the world's population is expected to be greater than sixty years of age. In concert with global aging of the population, neurodegenerative disorders have become the leading cause of disability with dementia now the seventh leading cause of death worldwide. Despite multi-faceted treatment approaches for disorders of cognition that include Alzheimer's disease and multiple sclerosis, present therapies ultimately cannot halt disease progression and eventually cognitive impairment continues unabated. Furthermore, co-morbidities, such as metabolic disorders with diabetes mellitus, also lack strategies to prevent disease progression. Given these clinical challenges for cognitive loss, innovative avenues of investigation that involve mammalian chronobiology with circadian rhythm clock genes and related pathways of aging, cellular senescence, oxidative stress, metabolic dysfunction, sleep fragmentation, apolipoprotein E, programmed cell death, silent mating type information regulation 2 homolog 1 (Saccharomyces cerevisiae), nicotinamide adenine dinucleotide, the gut microbiota, and glucagon-like peptide-1 receptor agonism may offer exceptional promise for forging new strategies for cognitive disease treatment. These pathways are intimately linked to circadian rhythm processes, are complex in generating biological outcomes, can broadly influence clinical translation of both short- and long-term considerations for cognitive disease care, and necessitate dissection of their precise regulatory mechanisms with the benefit from early diagnostic platforms as well as artificial intelligence and machine learning applications to foster translation of these pathways into effective clinical treatments.</t>
+          <t>Alzheimer's disease (AD) is the most common neurodegenerative disorder worldwide. Early diagnosis of AD is crucial for delaying disease progression and improving patients' quality of life. Blood biomarkers, particularly amyloid-beta (Aβ) and Tau proteins along with their phosphorylated isoforms, show advantages such as convenient sampling, minimal invasiveness, and excellent repeatability. However, the extremely low concentrations of AD biomarkers in blood impose stringent requirements on the sensitivity, specificity, and anti-interference capability of detection methods. Optical methods provide promising analytical platforms to address these challenges in view of their intrinsic merits of high sensitivity and selectivity; rapid response; and potential for miniaturization. This review systematically summarizes the latest advances in optical methods for the detection of the two core AD blood biomarkers (Aβ and Tau), covering techniques such as colorimetry, fluorescence, chemiluminescence, surface plasmon resonance (SPR), and surface-enhanced Raman scattering (SERS). The sensing principles, design strategies, and analytical performances of these methods are discussed, with special emphasis on different signal amplification strategies. In addition, several challenges and future prospects are provided with a primary focus on single-molecule detection, insufficient sensitivity and stability, lack of validation with large clinical cohorts, and absence of standardization. This review aims to provide researchers with guidance for the rational development of high-performance optical methods to achieve early diagnosis of AD.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>42767712</t>
+          <t>42645044</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Vulnerability in the womb: Charting the effects of prenatal cannabinoid exposure to mitigate developmental actions on dopamine metabolic capacities and circuits.</t>
+          <t>Overview in Electrochemical and Electrical Biosensors for Determining Blood Protein Biomarkers of Alzheimer's Disease.</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>International review of neurobiology</t>
+          <t>Biosensors</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -925,24 +925,24 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Prenatal cannabis exposure (PCE) is increasingly recognized as a major public health concern as cannabis use during pregnancy continues to rise worldwide. While early studies focused on cannabinoid receptor-mediated alterations in neurotransmission, emerging evidence indicates that PCE induces long-lasting developmental reprogramming affecting neural circuits, metabolism, and endocrine regulation. In this roadmap, we propose a shift from viewing PCE as a discrete synaptic disturbance to considering it a disorder of developmental coordination. We discuss how prenatal cannabinoid exposure may alter mesolimbic dopamine circuit maturation through the interaction of neuronal excitability, mitochondrial bioenergetics, and stress-related hormonal signaling. Particular attention is given to mitochondrial-circuit coupling in dopaminergic neurons and the potential role of mitochondrial cannabinoid receptors (mtCB1) in shaping long-term neuronal function. We further highlight the contribution of astrocytes, microglia, and neuroimmune processes in determining vulnerability or resilience trajectories. We propose that PCE generates latent neurobiological vulnerabilities that may emerge during adolescence or later life when challenged by environmental or physiological stressors. This framework provides new opportunities for early intervention, and prevention, while also offering insights into how early-life metabolic and mitochondrial dysfunction may contribute to lifelong brain vulnerability, including increased susceptibility to age-related neurodegenerative disorders such as Alzheimer's disease.</t>
+          <t>Early diagnosis of Alzheimer's disease (AD) can facilitate the establishment and implementation of therapeutic interventions. The currently used diagnosis methods for AD mainly include cerebrospinal fluid analysis and positron emission tomography imaging. Due to their high invasiveness, high cost, and limited accessibility, these technologies are difficult to meet the needs of large-scale population screening, grading diagnosis, and treatment, thereby limiting the popularization of early diagnosis of AD. The detection of blood biomarkers has become an important breakthrough in early screening and diagnosis of different diseases due to its non-invasive, low-cost, and easy-to-operation advantages. Recently, blood proteins such as amyloid-beta (Aβ), total and phosphorylated Tau, light chain neurofilaments (NFL), and glial fibrillary acidic protein (GFAP) have been considered promising biomarkers for the diagnosis of AD. However, there is currently no effective, minimally invasive, and easily accessible detection method for clinical diagnosis and risk prediction of AD. Electrochemical and electrical biosensors are highly sensitive, simple, fast, and cost-effective analytical tools for disease monitoring, drug development, and target detection. In this work, we comprehensively and systematically overview the progress of various electrochemical and electrical techniques for determining AD-related blood protein biomarkers, mainly including electrochemistry, electrochemiluminescence, photoelectrochemistry, quartz crystal microbalance, field-effect transistor, and organic electrochemical transistor. This work can provide guidance for researchers to develop novel electrochemical and electrical biosensors for early and accurate diagnosis of AD.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>42767254</t>
+          <t>42632212</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Burden of non-communicable diseases and their attributable risk factors in Africa from 1990 to 2023: a systematic analysis for the Global Burden of Disease Study 2023.</t>
+          <t>Rational design of halogen-substituted near-infrared fluorescent probes for butyrylcholinesterase: from drug screening to imaging and therapeutic evaluation in Alzheimer's disease.</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>The Lancet. Global health</t>
+          <t>Biosensors &amp; bioelectronics</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -952,24 +952,24 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>The rapid rise in the burden of non-communicable disease (NCDs) in African communities has resulted in a considerable mortality, disability, and economic burden. A comprehensive evaluation of incidence, deaths, disability-adjusted life-years (DALYs), and attributable risk factors related to NCDs by sex, and geographical location is essential for informing policy decisions aimed at controlling these diseases. This study used a comprehensive analysis based on the Global Burden of Diseases, Injuries, and Risk Factors Study (GBD) 2023 methodology to estimate the incidence, mortality, DALYs (estimated as the sum of years of life lost and years lived with disability [YLDs]), and attributable risk factors of NCDs in Africa. Data were systematically searched for and extracted from various sources, including vital registration, verbal autopsy, surveillance systems, police reports, censuses, surveys, minimally invasive tissue sampling, and sibling history. The analysis employed the Cause of Death Ensemble model, DisMod-MR 2.1, and spatiotemporal Gaussian process regression to estimate both fatal and non-fatal health metrics associated with NCDs in Africa overall, and by region and country. In 2023, NCDs in Africa accounted for an estimated 2·33 billion (95% uncertainty interval 2·22-2·50) incident cases, 4·70 million (4·47-4·93) deaths, and 263 million (234-293) DALYs. Although absolute numbers increased between 1990 and 2023, age-standardised rates (per 100 000 population) decreased modestly: incidence rate by 2·7% (0·2-5·0), mortality rate by 9·0% (2·5-15·5), and DALY rate by 6·4% (1·2-12·0). The five leading Level 3 causes of death in Africa in 2023 were ischaemic heart disease (801 000 [653 000-965 000]), stroke (700 000 [544 000-863 000]), chronic kidney disease (293 000 [224 000-359 000], hypertensive heart disease (246 000 [170 000-337 000]), and diabetes (245 000 [190 000-314 000]) for all sexes and ages. Leading Level 2 causes of YLDs were mental disorders (30·9 million [22·0-42·2]) and musculoskeletal disorders (17·1 million [12·5-22·7]). Overall, 35·1% (32·4-38·2) of DALYs and 57·4% (54·2-60·4) of deaths due to NCDs were attributable to the 88 GBD 2023 risk factors. High systolic blood pressure contributed the largest proportion at 26·2% (21·6-30·9) of all NCD deaths in Africa, followed by dietary risks (14·7% [5·1-21·6]) and air pollution (14·2% [11·6-16·9]). Our findings underscore the complex and evolving nature of the NCD burden in Africa, where modest declines in age-standardised mortality and DALY rates since 1990 have been substantially offset by rising absolute counts of deaths and DALYs-a paradox driven predominantly by rapid population growth and demographic changes. That more than half of all NCD deaths and over a third of DALYs remain attributable to modifiable risk factors-principally high systolic blood pressure, dietary risks, and air pollution-suggests that a substantial and actionable proportion of this burden is preventable through available and effective interventions, carrying urgent implications for African governments, ministries of health, and global health partners, who must take decisive action to meet health commitments. Gates Foundation.</t>
+          <t>Monitoring butyrylcholinesterase (BuChE) activity is crucial for tracking Alzheimer's disease (AD) progression and evaluating therapeutics; however, high-performance near-infrared (NIR) probes with rapid response and clear design principles remain scarce. Here, we report a series of dicyanoisophorone-based NIR fluorescent probes engineered via a "halogen effect" to systematically tune reactivity toward BuChE. Through spectroscopic screening, the CF</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>42767135</t>
+          <t>42618102</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Elucidating the molecular nexus between dental developmental anomalies and chronic inflammatory diseases: A computational systems biology analysis of genomic sequence homology using matrix factorization.</t>
+          <t>A dual-enhanced magnetically separable SERS strategy enabled by Fe</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Computational biology and chemistry</t>
+          <t>Analytica chimica acta</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -979,7 +979,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>This entirely in silico, exploratory study investigates potential sequence-level links between periodontal disease, developmental dental anomalies such as molar-incisor hypomineralization (MIH), and selected systemic conditions including leukemias, amyotrophic lateral sclerosis, and Alzheimer's disease. To identify annotation-independent signatures, we applied Non-negative Matrix Tri-Factorization (NMTF) to k-mer/tf-idf representations of disease-associated gene and protein sequences compiled from OMIM, GeneCards, and PubMed for eleven curated disease groups; similarity values denote the proportion of the total between-cluster interaction (S-matrix) captured by a cluster. To guard against trivial explanations, we applied a composition-preserving sequence-shuffling test of the similarity magnitude and a degree-preserving (curveball) permutation test of the disease co-clustering that accounts for the dependence introduced by isoform records and shared genes, repeating the latter across a 1890-configuration parameter grid. At the gene level the dominant cluster was governed by the largest disease group (MIH) rather than by disease identity, whereas at the protein level periodontitis, dental anomalies, and leukemia subtypes co-clustered. The magnitude of the shares did not exceed a composition-preserving null (gene p=0.66; protein p=0.082), and under the degree-preserving null co-clustering was not significant at the gene level (p=0.36) but was significant, modest, and grid-robust at the protein level (p=0.033); canonical k-mer and coding-sequence controls confirmed that the gene-level weakness is intrinsic to nucleotide k-mers. These results delineate the protein level as the informative scale for annotation-independent cross-disease screening and identify the dental-leukemia axis as the candidate relationship for targeted follow-up. The findings are hypothesis-generating: the disease-associated gene sets were compiled with a non-systematic, literature-guided procedure, magnitudes do not exceed composition baselines, neither experimental or clinical validation nor quantitative benchmarking against alternative computational frameworks was performed, and any translational implication requires future validation.</t>
+          <t>The accurate detection of highly specific biomarkers like phosphorylated tau217 (p-tau217) is a prerequisite for realizing the early diagnosis of Alzheimer' s disease. However, the reliable monitoring of p-tau217 is still prohibited by its extremely low abundance in complex biological fluids with significant interference. Herein, we propose a magnetically separable SERS-active sandwich immunosensor for the ultrasensitive detection of p-tau217. This design utilizes Fe This work establishes an ultrasensitive and magnetically separable SERS platform for the trace detection of p-tau217, which highlights the broad potential of synergizing hierarchical magnetic substrates with mesoporous metal-organic framework probes in clinical diagnostics.</t>
         </is>
       </c>
     </row>

</xml_diff>